<commit_message>
Use actual AUD/USD rate (0.6946); payback ~17 years
</commit_message>
<xml_diff>
--- a/data/rig-power-cost.xlsx
+++ b/data/rig-power-cost.xlsx
@@ -45,7 +45,7 @@
     <t xml:space="preserve">AUD per 1 USD</t>
   </si>
   <si>
-    <t xml:space="preserve">Approximate. Check the actual rate on the day you post.</t>
+    <t xml:space="preserve">1 AUD = 0.6946 USD (last close before 18 Oct 2026, tradingeconomics.com)</t>
   </si>
   <si>
     <t xml:space="preserve">Same model rented: output (US$/M tokens)</t>
@@ -853,7 +853,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="7" t="n">
-        <v>1.5</v>
+        <v>1.4397</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>7</v>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G5" s="26" t="n">
         <f aca="false">IFERROR(F5/Assumptions!$B$5,"")</f>
-        <v>0.471029446647013</v>
+        <v>0.490757914822893</v>
       </c>
       <c r="H5" s="15" t="s">
         <v>55</v>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="G6" s="26" t="n">
         <f aca="false">IFERROR(F6/Assumptions!$B$5,"")</f>
-        <v>0.756015435035416</v>
+        <v>0.787680178199017</v>
       </c>
       <c r="H6" s="15" t="s">
         <v>57</v>
@@ -1253,7 +1253,7 @@
       <c r="E7" s="24"/>
       <c r="F7" s="25" t="n">
         <f aca="false">G7*Assumptions!$B$5</f>
-        <v>1.2</v>
+        <v>1.15176</v>
       </c>
       <c r="G7" s="26" t="n">
         <f aca="false">Assumptions!B6</f>
@@ -1273,7 +1273,7 @@
       <c r="E8" s="24"/>
       <c r="F8" s="25" t="n">
         <f aca="false">G8*Assumptions!$B$5</f>
-        <v>7.5</v>
+        <v>7.1985</v>
       </c>
       <c r="G8" s="26" t="n">
         <f aca="false">Assumptions!B8</f>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="G11" s="26" t="n">
         <f aca="false">IFERROR(F11/Assumptions!$B$5,"")</f>
-        <v>0.0200727237210014</v>
+        <v>0.0209134441769134</v>
       </c>
       <c r="H11" s="15" t="s">
         <v>63</v>
@@ -1330,7 +1330,7 @@
       <c r="E12" s="24"/>
       <c r="F12" s="25" t="n">
         <f aca="false">G12*Assumptions!$B$5</f>
-        <v>0.18</v>
+        <v>0.172764</v>
       </c>
       <c r="G12" s="26" t="n">
         <f aca="false">Assumptions!B7</f>
@@ -1350,7 +1350,7 @@
       <c r="E13" s="24"/>
       <c r="F13" s="25" t="n">
         <f aca="false">G13*Assumptions!$B$5</f>
-        <v>1.5</v>
+        <v>1.4397</v>
       </c>
       <c r="G13" s="26" t="n">
         <f aca="false">Assumptions!B9</f>
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B17" s="27" t="n">
         <f aca="false">F7/F5</f>
-        <v>1.6984076169648</v>
+        <v>1.63013163076281</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>68</v>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B18" s="27" t="n">
         <f aca="false">F8/F5</f>
-        <v>10.61504760603</v>
+        <v>10.1883226922676</v>
       </c>
       <c r="C18" s="6"/>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="B19" s="27" t="n">
         <f aca="false">F12/F11</f>
-        <v>5.978261927376</v>
+        <v>5.73793579789548</v>
       </c>
       <c r="C19" s="6"/>
     </row>
@@ -1413,7 +1413,7 @@
       </c>
       <c r="B20" s="27" t="n">
         <f aca="false">F13/F11</f>
-        <v>49.8188493948</v>
+        <v>47.816131649129</v>
       </c>
       <c r="C20" s="6"/>
     </row>

</xml_diff>